<commit_message>
Met à jour les fichiers d'exemple avec le nouveau champ definition_local_km
</commit_message>
<xml_diff>
--- a/web/static/documents/achats_id_fichier_exemple_ma_cantine.xlsx
+++ b/web/static/documents/achats_id_fichier_exemple_ma_cantine.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t xml:space="preserve">cantine_id</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">definition_local</t>
   </si>
   <si>
+    <t xml:space="preserve">definition_local_km</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pommes, rouges</t>
   </si>
   <si>
@@ -86,6 +89,9 @@
   </si>
   <si>
     <t xml:space="preserve">11.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KM</t>
   </si>
 </sst>
 </file>
@@ -161,13 +167,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -305,7 +315,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.63"/>
@@ -316,11 +326,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="29.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18.9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="22.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -353,6 +364,9 @@
       </c>
       <c r="K1" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -360,34 +374,34 @@
         <v>949</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>46144</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="G2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -395,23 +409,30 @@
         <v>949</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>46144</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="0"/>
-      <c r="K3" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="G3" s="5"/>
+      <c r="J3" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
fix(Imports): Achats: corrige la colonne "definition_local_km" dans les nouveaux imports (#6896)
</commit_message>
<xml_diff>
--- a/web/static/documents/achats_id_fichier_exemple_ma_cantine.xlsx
+++ b/web/static/documents/achats_id_fichier_exemple_ma_cantine.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t xml:space="preserve">cantine_id</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">definition_local</t>
   </si>
   <si>
+    <t xml:space="preserve">definition_local_km</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pommes, rouges</t>
   </si>
   <si>
@@ -86,6 +89,9 @@
   </si>
   <si>
     <t xml:space="preserve">11.90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KM</t>
   </si>
 </sst>
 </file>
@@ -170,7 +176,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -305,7 +311,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.63"/>
@@ -316,11 +322,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="29.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="18.9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -353,6 +360,9 @@
       </c>
       <c r="K1" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -360,34 +370,34 @@
         <v>949</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>46144</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -395,23 +405,30 @@
         <v>949</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>46144</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="4"/>
-      <c r="H3" s="0"/>
-      <c r="K3" s="2"/>
+      <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>